<commit_message>
chore(translation): add persisted assets Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/backend/seed/knowledge/资源库/记忆库/AI翻译语料写入Excel.xlsx
+++ b/backend/seed/knowledge/资源库/记忆库/AI翻译语料写入Excel.xlsx
@@ -1242,7 +1242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="43.25" customWidth="1" style="1" min="1" max="1"/>
@@ -1262,23 +1262,125 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="0" t="inlineStr">
         <is>
           <t>本软件对接的实验室管理系统要求如下</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>The requirements for the applicable laboratory management system are described below:</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="27" customHeight="1" s="2"/>
-    <row r="5" ht="27" customHeight="1" s="2"/>
-    <row r="6" ht="27" customHeight="1" s="2"/>
-    <row r="7" ht="27" customHeight="1" s="2"/>
-    <row r="9" ht="27" customHeight="1" s="2"/>
-    <row r="10" ht="27" customHeight="1" s="2"/>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>G99 测序仪支持多种规格芯片上机，芯片拍照前需要通过拍照识别芯片内置的标识来定位芯片的位置。</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="inlineStr">
+        <is>
+          <t>G99 Genetic Sequencer supports sequencing with different types of flow cells. It determines the position of a flow cell by photographing and identifying the built-in marker of the flow cell before capturing images of the flow cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="27" customHeight="1" s="2">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>此位置信息会受到不同规格芯片的的安装位置以及芯片晶圆切割的位置影响。</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="inlineStr">
+        <is>
+          <t>This position information is affected by the mounting positions of flow cells of different types and the wafer cutting positions of the flow cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="27" customHeight="1" s="2">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>此位置信息会受到不同规格芯片的的安装位置以及芯片晶圆切割的位置影响。</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="inlineStr">
+        <is>
+          <t>This position information is affected by the mounting positions of flow cells of different types and the wafer cutting positions of the flow cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="27" customHeight="1" s="2">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>多芯片融合的拍照起点定位，是结合不同的芯片拍照预设置的起点位置（参考起始点），采用随机放置的芯片预拍照，获取到不同芯片的图片识别的算法行列，投射在晶圆所有Fov排布的统一视场中进行融合校准。</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="inlineStr">
+        <is>
+          <t>The imaging starting point in multi-flow cell fusion scenario is positioned using the following manner: According to the pre-configured imaging starting positions (reference starting point) of different types of flow cells, pre-image randomly selected flow cells to obtain images of the flow cells, then identify the images to obtain the algorithmic row and column information, and project the row and column information into a unified FOV encompassing all FOV layouts on the wafers of the flow cells for fusion calibration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="27" customHeight="1" s="2">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>常见故障处理</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="inlineStr">
+        <is>
+          <t>FAQs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>（可选）查看任务进度</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>(Optional) Viewing the task progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="27" customHeight="1" s="2">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>（可选）查看任务进度</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>(Optional) View the task progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="27" customHeight="1" s="2">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>SBS标准微孔板</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>SBS standard microplate</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SBS标准微孔板</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>standard microplate</t>
+        </is>
+      </c>
+    </row>
     <row r="13" ht="27" customHeight="1" s="2"/>
     <row r="14" ht="27" customHeight="1" s="2"/>
     <row r="17" ht="27" customHeight="1" s="2"/>

</xml_diff>